<commit_message>
Fix electricity tariff calculation and update master sheet row index
</commit_message>
<xml_diff>
--- a/docs/ГИРА_1006теккаа2.xlsx
+++ b/docs/ГИРА_1006теккаа2.xlsx
@@ -1782,14 +1782,14 @@
         <v>10000</v>
       </c>
       <c r="N3" s="60" t="n">
-        <v>423</v>
+        <v>500</v>
       </c>
       <c r="O3" s="6">
         <f>N3-K3</f>
         <v/>
       </c>
       <c r="P3" s="12" t="n">
-        <v>234</v>
+        <v>10000</v>
       </c>
       <c r="Q3" s="60" t="n"/>
       <c r="R3" s="6">
@@ -2192,7 +2192,7 @@
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="72" t="n"/>
       <c r="P6" s="8" t="n">
-        <v>234</v>
+        <v>25</v>
       </c>
       <c r="Q6" s="2" t="n"/>
       <c r="R6" s="72" t="n"/>
@@ -2360,7 +2360,7 @@
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="72" t="n"/>
       <c r="P8" s="8" t="n">
-        <v>234</v>
+        <v>25</v>
       </c>
       <c r="Q8" s="2" t="n"/>
       <c r="R8" s="72" t="n"/>
@@ -2716,7 +2716,7 @@
         <v/>
       </c>
       <c r="P11" s="6" t="n">
-        <v>432</v>
+        <v>80000</v>
       </c>
       <c r="Q11" s="2" t="n"/>
       <c r="R11" s="6">
@@ -11252,14 +11252,14 @@
         <v/>
       </c>
       <c r="N9" s="21" t="n">
-        <v>234</v>
+        <v>1000</v>
       </c>
       <c r="O9" s="22">
         <f>N9-K9</f>
         <v/>
       </c>
       <c r="P9" s="23" t="n">
-        <v>421</v>
+        <v>1500</v>
       </c>
       <c r="Q9" s="21" t="n"/>
       <c r="R9" s="22">

</xml_diff>

<commit_message>
fix(aiogram): add support for filename in FSInputFile and update _core to use it
</commit_message>
<xml_diff>
--- a/docs/ГИРА_1006теккаа2.xlsx
+++ b/docs/ГИРА_1006теккаа2.xlsx
@@ -1782,7 +1782,7 @@
         <v>10000</v>
       </c>
       <c r="N3" s="60" t="n">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="O3" s="6">
         <f>N3-K3</f>
@@ -2716,7 +2716,7 @@
         <v/>
       </c>
       <c r="P11" s="6" t="n">
-        <v>80000</v>
+        <v>15000</v>
       </c>
       <c r="Q11" s="2" t="n"/>
       <c r="R11" s="6">
@@ -11252,14 +11252,14 @@
         <v/>
       </c>
       <c r="N9" s="21" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="O9" s="22">
         <f>N9-K9</f>
         <v/>
       </c>
       <c r="P9" s="23" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="Q9" s="21" t="n"/>
       <c r="R9" s="22">

</xml_diff>

<commit_message>
feat: add director_fio_genitive migration, update handlers and docs templates
</commit_message>
<xml_diff>
--- a/docs/ГИРА_1006теккаа2.xlsx
+++ b/docs/ГИРА_1006теккаа2.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K27.8" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K52.0" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K61.0" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K12.0" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1386,7 +1387,7 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>550</v>
+        <v>21441</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
@@ -1394,7 +1395,7 @@
         </is>
       </c>
       <c r="K2" s="4" t="n">
-        <v>10000</v>
+        <v>124124</v>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
@@ -1774,7 +1775,7 @@
         <v>20000</v>
       </c>
       <c r="K3" s="59" t="n">
-        <v>350</v>
+        <v>5.789096</v>
       </c>
       <c r="L3" s="6">
         <f>K3-H3</f>
@@ -2106,7 +2107,7 @@
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="59" t="n">
-        <v>40</v>
+        <v>24112</v>
       </c>
       <c r="L5" s="6" t="n"/>
       <c r="M5" s="6" t="n"/>
@@ -2276,7 +2277,7 @@
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="59" t="n">
-        <v>40</v>
+        <v>24112</v>
       </c>
       <c r="L7" s="6" t="n"/>
       <c r="M7" s="6" t="n"/>
@@ -3003,7 +3004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
   <cols>
     <col width="13.83203125" customWidth="1" min="1" max="1"/>
@@ -4631,6 +4632,69 @@
       <c r="V23" t="inlineStr">
         <is>
           <t>16.12.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2818222828</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ООО</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ОШИБКА</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>магазин</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>12</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>K12.0</t>
+        </is>
+      </c>
+      <c r="K24" s="86" t="n">
+        <v>45638</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>231323</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Нагимов</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Ранель</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Алмазович</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>12.12.3999</t>
         </is>
       </c>
     </row>
@@ -11517,7 +11581,7 @@
         <v/>
       </c>
       <c r="P9" s="23" t="n">
-        <v>453</v>
+        <v>421421</v>
       </c>
       <c r="Q9" s="21" t="n"/>
       <c r="R9" s="22">
@@ -12166,7 +12230,7 @@
       <c r="N12" s="24" t="n"/>
       <c r="O12" s="24" t="n"/>
       <c r="P12" s="25" t="n">
-        <v>345</v>
+        <v>24112</v>
       </c>
       <c r="Q12" s="24" t="n"/>
       <c r="R12" s="24" t="n"/>
@@ -12307,7 +12371,7 @@
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="16" t="n"/>
       <c r="P13" t="n">
-        <v>345</v>
+        <v>24112</v>
       </c>
     </row>
     <row r="14">
@@ -17343,7 +17407,7 @@
         <v/>
       </c>
       <c r="P9" s="23" t="n">
-        <v>12345</v>
+        <v>124124</v>
       </c>
       <c r="Q9" s="21" t="n"/>
       <c r="R9" s="22">
@@ -17992,7 +18056,7 @@
       <c r="N12" s="24" t="n"/>
       <c r="O12" s="24" t="n"/>
       <c r="P12" s="25" t="n">
-        <v>16</v>
+        <v>42112</v>
       </c>
       <c r="Q12" s="24" t="n"/>
       <c r="R12" s="24" t="n"/>
@@ -18133,7 +18197,7 @@
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="16" t="n"/>
       <c r="P13" t="n">
-        <v>12</v>
+        <v>241124</v>
       </c>
     </row>
     <row r="14">
@@ -21044,4 +21108,2903 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CD16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="25.33203125" customWidth="1" min="2" max="2"/>
+    <col width="25.5" customWidth="1" style="1" min="3" max="3"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.33203125" customWidth="1" min="5" max="5"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
+    <col width="11.33203125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12.5" customWidth="1" min="8" max="8"/>
+    <col width="10.83203125" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
+    <col width="13.6640625" customWidth="1" style="1" min="10" max="10"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="12" max="12"/>
+    <col width="20.5" customWidth="1" style="1" min="13" max="13"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="15" max="15"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="16" max="16"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="18" max="18"/>
+    <col width="12" customWidth="1" style="1" min="19" max="19"/>
+    <col width="8.83203125" bestFit="1" customWidth="1" min="20" max="20"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="21" max="22"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="23" max="23"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="24" max="25"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="26" max="26"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="27" max="28"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="29" max="29"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="30" max="31"/>
+    <col width="8.83203125" bestFit="1" customWidth="1" min="32" max="32"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="33" max="34"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="35" max="35"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="36" max="37"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="38" max="38"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="39" max="40"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="41" max="41"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="42" max="43"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="44" max="44"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="1" min="45" max="46"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="47" max="47"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="48" max="49"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="50" max="50"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="51" max="52"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="53" max="53"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="54" max="55"/>
+    <col width="8.83203125" bestFit="1" customWidth="1" min="56" max="56"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="57" max="64"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="65" max="65"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="66" max="67"/>
+    <col width="8.83203125" bestFit="1" customWidth="1" min="68" max="68"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="69" max="70"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="71" max="71"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="72" max="73"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="74" max="74"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="75" max="76"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="77" max="77"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="78" max="79"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="80" max="80"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="81" max="82"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>ИНН</t>
+        </is>
+      </c>
+      <c r="B1" s="33">
+        <f>Реестр!D3</f>
+        <v/>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Месяц</t>
+        </is>
+      </c>
+      <c r="D1" s="19" t="n">
+        <v>45962</v>
+      </c>
+      <c r="E1" s="19" t="n">
+        <v>45992</v>
+      </c>
+      <c r="F1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="G1" s="75" t="n">
+        <v>45962</v>
+      </c>
+      <c r="H1" s="19" t="n">
+        <v>46023</v>
+      </c>
+      <c r="I1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="J1" s="75" t="n">
+        <v>45992</v>
+      </c>
+      <c r="K1" s="19" t="n">
+        <v>46054</v>
+      </c>
+      <c r="L1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="M1" s="75" t="n">
+        <v>46023</v>
+      </c>
+      <c r="N1" s="19" t="n">
+        <v>46082</v>
+      </c>
+      <c r="O1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="P1" s="75" t="n">
+        <v>46054</v>
+      </c>
+      <c r="Q1" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="R1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="S1" s="75" t="n">
+        <v>46082</v>
+      </c>
+      <c r="T1" s="19" t="n">
+        <v>46143</v>
+      </c>
+      <c r="U1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="V1" s="75" t="n">
+        <v>46113</v>
+      </c>
+      <c r="W1" s="19" t="n">
+        <v>46174</v>
+      </c>
+      <c r="X1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="Y1" s="75" t="n">
+        <v>46143</v>
+      </c>
+      <c r="Z1" s="19" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AA1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AB1" s="75" t="n">
+        <v>46174</v>
+      </c>
+      <c r="AC1" s="19" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AD1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AE1" s="75" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AF1" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AG1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AH1" s="75" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AI1" s="19" t="n">
+        <v>46296</v>
+      </c>
+      <c r="AJ1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AK1" s="75" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AL1" s="19" t="n">
+        <v>46327</v>
+      </c>
+      <c r="AM1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AN1" s="75" t="n">
+        <v>46296</v>
+      </c>
+      <c r="AO1" s="19" t="n">
+        <v>46357</v>
+      </c>
+      <c r="AP1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AQ1" s="75" t="n">
+        <v>46327</v>
+      </c>
+      <c r="AR1" s="19" t="n">
+        <v>46388</v>
+      </c>
+      <c r="AS1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AT1" s="75" t="n">
+        <v>46357</v>
+      </c>
+      <c r="AU1" s="19" t="n">
+        <v>46419</v>
+      </c>
+      <c r="AV1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AW1" s="75" t="n">
+        <v>46388</v>
+      </c>
+      <c r="AX1" s="19" t="n">
+        <v>46447</v>
+      </c>
+      <c r="AY1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="AZ1" s="75" t="n">
+        <v>46419</v>
+      </c>
+      <c r="BA1" s="19" t="n">
+        <v>46478</v>
+      </c>
+      <c r="BB1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BC1" s="75" t="n">
+        <v>46447</v>
+      </c>
+      <c r="BD1" s="19" t="n">
+        <v>46508</v>
+      </c>
+      <c r="BE1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BF1" s="75" t="n">
+        <v>46478</v>
+      </c>
+      <c r="BG1" s="19" t="n">
+        <v>46539</v>
+      </c>
+      <c r="BH1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BI1" s="75" t="n">
+        <v>46508</v>
+      </c>
+      <c r="BJ1" s="19" t="n">
+        <v>46569</v>
+      </c>
+      <c r="BK1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BL1" s="75" t="n">
+        <v>46539</v>
+      </c>
+      <c r="BM1" s="19" t="n">
+        <v>46600</v>
+      </c>
+      <c r="BN1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BO1" s="75" t="n">
+        <v>46569</v>
+      </c>
+      <c r="BP1" s="19" t="n">
+        <v>46631</v>
+      </c>
+      <c r="BQ1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BR1" s="75" t="n">
+        <v>46600</v>
+      </c>
+      <c r="BS1" s="19" t="n">
+        <v>46661</v>
+      </c>
+      <c r="BT1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BU1" s="75" t="n">
+        <v>46631</v>
+      </c>
+      <c r="BV1" s="19" t="n">
+        <v>46692</v>
+      </c>
+      <c r="BW1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="BX1" s="75" t="n">
+        <v>46661</v>
+      </c>
+      <c r="BY1" s="19" t="n">
+        <v>46722</v>
+      </c>
+      <c r="BZ1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="CA1" s="75" t="n">
+        <v>46692</v>
+      </c>
+      <c r="CB1" s="19" t="n">
+        <v>46753</v>
+      </c>
+      <c r="CC1" s="74" t="inlineStr">
+        <is>
+          <t>Потребл.</t>
+        </is>
+      </c>
+      <c r="CD1" s="75" t="n">
+        <v>46722</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>Кадастр</t>
+        </is>
+      </c>
+      <c r="B2" s="33">
+        <f>Реестр!B3</f>
+        <v/>
+      </c>
+      <c r="C2" s="74" t="n"/>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="H2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="I2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="M2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="N2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="O2" s="17" t="inlineStr">
+        <is>
+          <t>знач</t>
+        </is>
+      </c>
+      <c r="P2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="Q2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="R2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="S2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="T2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="U2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="V2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="W2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="X2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="Y2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="Z2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AA2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AB2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AC2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AD2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AE2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AF2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AG2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AH2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AI2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AJ2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AK2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AL2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AM2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AN2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AO2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AP2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AQ2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AR2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AS2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AT2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AU2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AV2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AW2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="AX2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AY2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="AZ2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BA2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BB2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BC2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BD2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BE2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BF2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BG2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BH2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BI2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BJ2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BK2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BL2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BM2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BN2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BO2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BP2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BQ2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BR2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BS2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BT2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BU2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BV2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BW2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BX2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="BY2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="BZ2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="CA2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="CB2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="CC2" s="17" t="inlineStr">
+        <is>
+          <t>знач.</t>
+        </is>
+      </c>
+      <c r="CD2" s="17" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="33" t="inlineStr">
+        <is>
+          <t>Арендатор</t>
+        </is>
+      </c>
+      <c r="B3" s="34">
+        <f>Реестр!F3</f>
+        <v/>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Электричество</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="22">
+        <f>E3-D3</f>
+        <v/>
+      </c>
+      <c r="G3" s="23">
+        <f>F3*G4</f>
+        <v/>
+      </c>
+      <c r="H3" s="21" t="n"/>
+      <c r="I3" s="22">
+        <f>H3-E3</f>
+        <v/>
+      </c>
+      <c r="J3" s="23">
+        <f>I3*J4</f>
+        <v/>
+      </c>
+      <c r="K3" s="21" t="n"/>
+      <c r="L3" s="22">
+        <f>K3-H3</f>
+        <v/>
+      </c>
+      <c r="M3" s="23">
+        <f>L3*M4</f>
+        <v/>
+      </c>
+      <c r="N3" s="21" t="n"/>
+      <c r="O3" s="22">
+        <f>N3-K3</f>
+        <v/>
+      </c>
+      <c r="P3" s="23">
+        <f>O3*P4</f>
+        <v/>
+      </c>
+      <c r="Q3" s="21" t="n"/>
+      <c r="R3" s="22">
+        <f>Q3-N3</f>
+        <v/>
+      </c>
+      <c r="S3" s="23">
+        <f>R3*S4</f>
+        <v/>
+      </c>
+      <c r="T3" s="21" t="n"/>
+      <c r="U3" s="22">
+        <f>T3-Q3</f>
+        <v/>
+      </c>
+      <c r="V3" s="23">
+        <f>U3*V4</f>
+        <v/>
+      </c>
+      <c r="W3" s="21" t="n"/>
+      <c r="X3" s="22">
+        <f>W3-T3</f>
+        <v/>
+      </c>
+      <c r="Y3" s="23">
+        <f>X3*Y4</f>
+        <v/>
+      </c>
+      <c r="Z3" s="21" t="n"/>
+      <c r="AA3" s="22">
+        <f>Z3-W3</f>
+        <v/>
+      </c>
+      <c r="AB3" s="23">
+        <f>AA3*AB4</f>
+        <v/>
+      </c>
+      <c r="AC3" s="21" t="n"/>
+      <c r="AD3" s="22">
+        <f>AC3-Z3</f>
+        <v/>
+      </c>
+      <c r="AE3" s="23">
+        <f>AD3*AE4</f>
+        <v/>
+      </c>
+      <c r="AF3" s="21" t="n"/>
+      <c r="AG3" s="22">
+        <f>AF3-AC3</f>
+        <v/>
+      </c>
+      <c r="AH3" s="23">
+        <f>AG3*AH4</f>
+        <v/>
+      </c>
+      <c r="AI3" s="21" t="n"/>
+      <c r="AJ3" s="22">
+        <f>AI3-AF3</f>
+        <v/>
+      </c>
+      <c r="AK3" s="23">
+        <f>AJ3*AK4</f>
+        <v/>
+      </c>
+      <c r="AL3" s="21" t="n"/>
+      <c r="AM3" s="22">
+        <f>AL3-AI3</f>
+        <v/>
+      </c>
+      <c r="AN3" s="23">
+        <f>AM3*AN4</f>
+        <v/>
+      </c>
+      <c r="AO3" s="21" t="n"/>
+      <c r="AP3" s="22">
+        <f>AO3-AL3</f>
+        <v/>
+      </c>
+      <c r="AQ3" s="23">
+        <f>AP3*AQ4</f>
+        <v/>
+      </c>
+      <c r="AR3" s="21" t="n"/>
+      <c r="AS3" s="22">
+        <f>AR3-AO3</f>
+        <v/>
+      </c>
+      <c r="AT3" s="23">
+        <f>AS3*AT4</f>
+        <v/>
+      </c>
+      <c r="AU3" s="21" t="n"/>
+      <c r="AV3" s="22">
+        <f>AU3-AR3</f>
+        <v/>
+      </c>
+      <c r="AW3" s="23">
+        <f>AV3*AW4</f>
+        <v/>
+      </c>
+      <c r="AX3" s="21" t="n"/>
+      <c r="AY3" s="22">
+        <f>AX3-AU3</f>
+        <v/>
+      </c>
+      <c r="AZ3" s="23">
+        <f>AY3*AZ4</f>
+        <v/>
+      </c>
+      <c r="BA3" s="21" t="n"/>
+      <c r="BB3" s="22">
+        <f>BA3-AX3</f>
+        <v/>
+      </c>
+      <c r="BC3" s="23">
+        <f>BB3*BC4</f>
+        <v/>
+      </c>
+      <c r="BD3" s="21" t="n"/>
+      <c r="BE3" s="22">
+        <f>BD3-BA3</f>
+        <v/>
+      </c>
+      <c r="BF3" s="23">
+        <f>BE3*BF4</f>
+        <v/>
+      </c>
+      <c r="BG3" s="21" t="n"/>
+      <c r="BH3" s="22">
+        <f>BG3-BD3</f>
+        <v/>
+      </c>
+      <c r="BI3" s="23">
+        <f>BH3*BI4</f>
+        <v/>
+      </c>
+      <c r="BJ3" s="21" t="n"/>
+      <c r="BK3" s="22">
+        <f>BJ3-BG3</f>
+        <v/>
+      </c>
+      <c r="BL3" s="23">
+        <f>BK3*BL4</f>
+        <v/>
+      </c>
+      <c r="BM3" s="21" t="n"/>
+      <c r="BN3" s="22">
+        <f>BM3-BJ3</f>
+        <v/>
+      </c>
+      <c r="BO3" s="23">
+        <f>BN3*BO4</f>
+        <v/>
+      </c>
+      <c r="BP3" s="21" t="n"/>
+      <c r="BQ3" s="22">
+        <f>BP3-BM3</f>
+        <v/>
+      </c>
+      <c r="BR3" s="23">
+        <f>BQ3*BR4</f>
+        <v/>
+      </c>
+      <c r="BS3" s="21" t="n"/>
+      <c r="BT3" s="22">
+        <f>BS3-BP3</f>
+        <v/>
+      </c>
+      <c r="BU3" s="23">
+        <f>BT3*BU4</f>
+        <v/>
+      </c>
+      <c r="BV3" s="21" t="n"/>
+      <c r="BW3" s="22">
+        <f>BV3-BS3</f>
+        <v/>
+      </c>
+      <c r="BX3" s="23">
+        <f>BW3*BX4</f>
+        <v/>
+      </c>
+      <c r="BY3" s="21" t="n"/>
+      <c r="BZ3" s="22">
+        <f>BY3-BV3</f>
+        <v/>
+      </c>
+      <c r="CA3" s="23">
+        <f>BZ3*CA4</f>
+        <v/>
+      </c>
+      <c r="CB3" s="21" t="n"/>
+      <c r="CC3" s="22">
+        <f>CB3-BY3</f>
+        <v/>
+      </c>
+      <c r="CD3" s="23">
+        <f>CC3*CD4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>Площадь</t>
+        </is>
+      </c>
+      <c r="B4" s="34">
+        <f>Реестр!H3</f>
+        <v/>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Электричество тариф</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="24" t="n"/>
+      <c r="G4" s="25">
+        <f>'0. ГИРА'!G4</f>
+        <v/>
+      </c>
+      <c r="H4" s="24" t="n"/>
+      <c r="I4" s="24" t="n"/>
+      <c r="J4" s="25">
+        <f>'0. ГИРА'!J4</f>
+        <v/>
+      </c>
+      <c r="K4" s="24" t="n"/>
+      <c r="L4" s="24" t="n"/>
+      <c r="M4" s="25">
+        <f>'0. ГИРА'!M4</f>
+        <v/>
+      </c>
+      <c r="N4" s="24" t="n"/>
+      <c r="O4" s="24" t="n"/>
+      <c r="P4" s="25">
+        <f>'0. ГИРА'!P4</f>
+        <v/>
+      </c>
+      <c r="Q4" s="24" t="n"/>
+      <c r="R4" s="24" t="n"/>
+      <c r="S4" s="25">
+        <f>'0. ГИРА'!S4</f>
+        <v/>
+      </c>
+      <c r="T4" s="24" t="n"/>
+      <c r="U4" s="24" t="n"/>
+      <c r="V4" s="25">
+        <f>'0. ГИРА'!V4</f>
+        <v/>
+      </c>
+      <c r="W4" s="24" t="n"/>
+      <c r="X4" s="24" t="n"/>
+      <c r="Y4" s="25">
+        <f>'0. ГИРА'!Y4</f>
+        <v/>
+      </c>
+      <c r="Z4" s="24" t="n"/>
+      <c r="AA4" s="24" t="n"/>
+      <c r="AB4" s="25">
+        <f>'0. ГИРА'!AB4</f>
+        <v/>
+      </c>
+      <c r="AC4" s="24" t="n"/>
+      <c r="AD4" s="24" t="n"/>
+      <c r="AE4" s="25">
+        <f>'0. ГИРА'!AE4</f>
+        <v/>
+      </c>
+      <c r="AF4" s="24" t="n"/>
+      <c r="AG4" s="24" t="n"/>
+      <c r="AH4" s="25">
+        <f>'0. ГИРА'!AH4</f>
+        <v/>
+      </c>
+      <c r="AI4" s="24" t="n"/>
+      <c r="AJ4" s="24" t="n"/>
+      <c r="AK4" s="25">
+        <f>'0. ГИРА'!AK4</f>
+        <v/>
+      </c>
+      <c r="AL4" s="24" t="n"/>
+      <c r="AM4" s="24" t="n"/>
+      <c r="AN4" s="25">
+        <f>'0. ГИРА'!AN4</f>
+        <v/>
+      </c>
+      <c r="AO4" s="24" t="n"/>
+      <c r="AP4" s="24" t="n"/>
+      <c r="AQ4" s="25">
+        <f>'0. ГИРА'!AQ4</f>
+        <v/>
+      </c>
+      <c r="AR4" s="24" t="n"/>
+      <c r="AS4" s="24" t="n"/>
+      <c r="AT4" s="25">
+        <f>'0. ГИРА'!AT4</f>
+        <v/>
+      </c>
+      <c r="AU4" s="24" t="n"/>
+      <c r="AV4" s="24" t="n"/>
+      <c r="AW4" s="25">
+        <f>'0. ГИРА'!AW4</f>
+        <v/>
+      </c>
+      <c r="AX4" s="24" t="n"/>
+      <c r="AY4" s="24" t="n"/>
+      <c r="AZ4" s="25">
+        <f>'0. ГИРА'!AZ4</f>
+        <v/>
+      </c>
+      <c r="BA4" s="24" t="n"/>
+      <c r="BB4" s="24" t="n"/>
+      <c r="BC4" s="25">
+        <f>'0. ГИРА'!BC4</f>
+        <v/>
+      </c>
+      <c r="BD4" s="24" t="n"/>
+      <c r="BE4" s="24" t="n"/>
+      <c r="BF4" s="25">
+        <f>'0. ГИРА'!BF4</f>
+        <v/>
+      </c>
+      <c r="BG4" s="24" t="n"/>
+      <c r="BH4" s="24" t="n"/>
+      <c r="BI4" s="25">
+        <f>'0. ГИРА'!BI4</f>
+        <v/>
+      </c>
+      <c r="BJ4" s="24" t="n"/>
+      <c r="BK4" s="24" t="n"/>
+      <c r="BL4" s="25">
+        <f>'0. ГИРА'!BL4</f>
+        <v/>
+      </c>
+      <c r="BM4" s="24" t="n"/>
+      <c r="BN4" s="24" t="n"/>
+      <c r="BO4" s="25">
+        <f>'0. ГИРА'!BO4</f>
+        <v/>
+      </c>
+      <c r="BP4" s="24" t="n"/>
+      <c r="BQ4" s="24" t="n"/>
+      <c r="BR4" s="25">
+        <f>'0. ГИРА'!BR4</f>
+        <v/>
+      </c>
+      <c r="BS4" s="24" t="n"/>
+      <c r="BT4" s="24" t="n"/>
+      <c r="BU4" s="25">
+        <f>'0. ГИРА'!BU4</f>
+        <v/>
+      </c>
+      <c r="BV4" s="24" t="n"/>
+      <c r="BW4" s="24" t="n"/>
+      <c r="BX4" s="25">
+        <f>'0. ГИРА'!BX4</f>
+        <v/>
+      </c>
+      <c r="BY4" s="24" t="n"/>
+      <c r="BZ4" s="24" t="n"/>
+      <c r="CA4" s="25">
+        <f>'0. ГИРА'!CA4</f>
+        <v/>
+      </c>
+      <c r="CB4" s="24" t="n"/>
+      <c r="CC4" s="24" t="n"/>
+      <c r="CD4" s="25">
+        <f>'0. ГИРА'!CD4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="36" t="n"/>
+      <c r="B5" s="36" t="n"/>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Водоканал холодная вода</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="22">
+        <f>E5-D5</f>
+        <v/>
+      </c>
+      <c r="G5" s="23">
+        <f>G6*F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="21" t="n"/>
+      <c r="I5" s="22">
+        <f>H5-E5</f>
+        <v/>
+      </c>
+      <c r="J5" s="23">
+        <f>J6*I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="21" t="n"/>
+      <c r="L5" s="22">
+        <f>K5-H5</f>
+        <v/>
+      </c>
+      <c r="M5" s="23">
+        <f>M6*L5</f>
+        <v/>
+      </c>
+      <c r="N5" s="21" t="n"/>
+      <c r="O5" s="22">
+        <f>N5-K5</f>
+        <v/>
+      </c>
+      <c r="P5" s="23">
+        <f>P6*O5</f>
+        <v/>
+      </c>
+      <c r="Q5" s="21" t="n"/>
+      <c r="R5" s="22">
+        <f>Q5-N5</f>
+        <v/>
+      </c>
+      <c r="S5" s="23">
+        <f>S6*R5</f>
+        <v/>
+      </c>
+      <c r="T5" s="21" t="n"/>
+      <c r="U5" s="22">
+        <f>T5-Q5</f>
+        <v/>
+      </c>
+      <c r="V5" s="23">
+        <f>V6*U5</f>
+        <v/>
+      </c>
+      <c r="W5" s="21" t="n"/>
+      <c r="X5" s="22">
+        <f>W5-T5</f>
+        <v/>
+      </c>
+      <c r="Y5" s="23">
+        <f>Y6*X5</f>
+        <v/>
+      </c>
+      <c r="Z5" s="21" t="n"/>
+      <c r="AA5" s="22">
+        <f>Z5-W5</f>
+        <v/>
+      </c>
+      <c r="AB5" s="23">
+        <f>AB6*AA5</f>
+        <v/>
+      </c>
+      <c r="AC5" s="21" t="n"/>
+      <c r="AD5" s="22">
+        <f>AC5-Z5</f>
+        <v/>
+      </c>
+      <c r="AE5" s="23">
+        <f>AE6*AD5</f>
+        <v/>
+      </c>
+      <c r="AF5" s="21" t="n"/>
+      <c r="AG5" s="22">
+        <f>AF5-AC5</f>
+        <v/>
+      </c>
+      <c r="AH5" s="23">
+        <f>AH6*AG5</f>
+        <v/>
+      </c>
+      <c r="AI5" s="21" t="n"/>
+      <c r="AJ5" s="22">
+        <f>AI5-AF5</f>
+        <v/>
+      </c>
+      <c r="AK5" s="23">
+        <f>AK6*AJ5</f>
+        <v/>
+      </c>
+      <c r="AL5" s="21" t="n"/>
+      <c r="AM5" s="22">
+        <f>AL5-AI5</f>
+        <v/>
+      </c>
+      <c r="AN5" s="23">
+        <f>AN6*AM5</f>
+        <v/>
+      </c>
+      <c r="AO5" s="21" t="n"/>
+      <c r="AP5" s="22">
+        <f>AO5-AL5</f>
+        <v/>
+      </c>
+      <c r="AQ5" s="23">
+        <f>AQ6*AP5</f>
+        <v/>
+      </c>
+      <c r="AR5" s="21" t="n"/>
+      <c r="AS5" s="22">
+        <f>AR5-AO5</f>
+        <v/>
+      </c>
+      <c r="AT5" s="23">
+        <f>AT6*AS5</f>
+        <v/>
+      </c>
+      <c r="AU5" s="21" t="n"/>
+      <c r="AV5" s="22">
+        <f>AU5-AR5</f>
+        <v/>
+      </c>
+      <c r="AW5" s="23">
+        <f>AW6*AV5</f>
+        <v/>
+      </c>
+      <c r="AX5" s="21" t="n"/>
+      <c r="AY5" s="22">
+        <f>AX5-AU5</f>
+        <v/>
+      </c>
+      <c r="AZ5" s="23">
+        <f>AZ6*AY5</f>
+        <v/>
+      </c>
+      <c r="BA5" s="21" t="n"/>
+      <c r="BB5" s="22">
+        <f>BA5-AX5</f>
+        <v/>
+      </c>
+      <c r="BC5" s="23">
+        <f>BC6*BB5</f>
+        <v/>
+      </c>
+      <c r="BD5" s="21" t="n"/>
+      <c r="BE5" s="22">
+        <f>BD5-BA5</f>
+        <v/>
+      </c>
+      <c r="BF5" s="23">
+        <f>BF6*BE5</f>
+        <v/>
+      </c>
+      <c r="BG5" s="21" t="n"/>
+      <c r="BH5" s="22">
+        <f>BG5-BD5</f>
+        <v/>
+      </c>
+      <c r="BI5" s="23">
+        <f>BI6*BH5</f>
+        <v/>
+      </c>
+      <c r="BJ5" s="21" t="n"/>
+      <c r="BK5" s="22">
+        <f>BJ5-BG5</f>
+        <v/>
+      </c>
+      <c r="BL5" s="23">
+        <f>BL6*BK5</f>
+        <v/>
+      </c>
+      <c r="BM5" s="21" t="n"/>
+      <c r="BN5" s="22">
+        <f>BM5-BJ5</f>
+        <v/>
+      </c>
+      <c r="BO5" s="23">
+        <f>BO6*BN5</f>
+        <v/>
+      </c>
+      <c r="BP5" s="21" t="n"/>
+      <c r="BQ5" s="22">
+        <f>BP5-BM5</f>
+        <v/>
+      </c>
+      <c r="BR5" s="23">
+        <f>BR6*BQ5</f>
+        <v/>
+      </c>
+      <c r="BS5" s="21" t="n"/>
+      <c r="BT5" s="22">
+        <f>BS5-BP5</f>
+        <v/>
+      </c>
+      <c r="BU5" s="23">
+        <f>BU6*BT5</f>
+        <v/>
+      </c>
+      <c r="BV5" s="21" t="n"/>
+      <c r="BW5" s="22">
+        <f>BV5-BS5</f>
+        <v/>
+      </c>
+      <c r="BX5" s="23">
+        <f>BX6*BW5</f>
+        <v/>
+      </c>
+      <c r="BY5" s="21" t="n"/>
+      <c r="BZ5" s="22">
+        <f>BY5-BV5</f>
+        <v/>
+      </c>
+      <c r="CA5" s="23">
+        <f>CA6*BZ5</f>
+        <v/>
+      </c>
+      <c r="CB5" s="21" t="n"/>
+      <c r="CC5" s="22">
+        <f>CB5-BY5</f>
+        <v/>
+      </c>
+      <c r="CD5" s="23">
+        <f>CD6*CC5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>Имя 1</t>
+        </is>
+      </c>
+      <c r="B6" s="34">
+        <f>Реестр!M3</f>
+        <v/>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Водоканал холодная Тариф</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="25">
+        <f>'0. ГИРА'!G6</f>
+        <v/>
+      </c>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="25">
+        <f>'0. ГИРА'!J6</f>
+        <v/>
+      </c>
+      <c r="K6" s="24" t="n"/>
+      <c r="L6" s="24" t="n"/>
+      <c r="M6" s="25">
+        <f>'0. ГИРА'!M6</f>
+        <v/>
+      </c>
+      <c r="N6" s="24" t="n"/>
+      <c r="O6" s="24" t="n"/>
+      <c r="P6" s="25">
+        <f>'0. ГИРА'!P6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="24" t="n"/>
+      <c r="R6" s="24" t="n"/>
+      <c r="S6" s="25">
+        <f>'0. ГИРА'!S6</f>
+        <v/>
+      </c>
+      <c r="T6" s="24" t="n"/>
+      <c r="U6" s="24" t="n"/>
+      <c r="V6" s="25">
+        <f>'0. ГИРА'!V6</f>
+        <v/>
+      </c>
+      <c r="W6" s="24" t="n"/>
+      <c r="X6" s="24" t="n"/>
+      <c r="Y6" s="25">
+        <f>'0. ГИРА'!Y6</f>
+        <v/>
+      </c>
+      <c r="Z6" s="24" t="n"/>
+      <c r="AA6" s="24" t="n"/>
+      <c r="AB6" s="25">
+        <f>'0. ГИРА'!AB6</f>
+        <v/>
+      </c>
+      <c r="AC6" s="24" t="n"/>
+      <c r="AD6" s="24" t="n"/>
+      <c r="AE6" s="25">
+        <f>'0. ГИРА'!AE6</f>
+        <v/>
+      </c>
+      <c r="AF6" s="24" t="n"/>
+      <c r="AG6" s="24" t="n"/>
+      <c r="AH6" s="25">
+        <f>'0. ГИРА'!AH6</f>
+        <v/>
+      </c>
+      <c r="AI6" s="24" t="n"/>
+      <c r="AJ6" s="24" t="n"/>
+      <c r="AK6" s="25">
+        <f>'0. ГИРА'!AK6</f>
+        <v/>
+      </c>
+      <c r="AL6" s="24" t="n"/>
+      <c r="AM6" s="24" t="n"/>
+      <c r="AN6" s="25">
+        <f>'0. ГИРА'!AN6</f>
+        <v/>
+      </c>
+      <c r="AO6" s="24" t="n"/>
+      <c r="AP6" s="24" t="n"/>
+      <c r="AQ6" s="25">
+        <f>'0. ГИРА'!AQ6</f>
+        <v/>
+      </c>
+      <c r="AR6" s="24" t="n"/>
+      <c r="AS6" s="24" t="n"/>
+      <c r="AT6" s="25">
+        <f>'0. ГИРА'!AT6</f>
+        <v/>
+      </c>
+      <c r="AU6" s="24" t="n"/>
+      <c r="AV6" s="24" t="n"/>
+      <c r="AW6" s="25">
+        <f>'0. ГИРА'!AW6</f>
+        <v/>
+      </c>
+      <c r="AX6" s="24" t="n"/>
+      <c r="AY6" s="24" t="n"/>
+      <c r="AZ6" s="25">
+        <f>'0. ГИРА'!AZ6</f>
+        <v/>
+      </c>
+      <c r="BA6" s="24" t="n"/>
+      <c r="BB6" s="24" t="n"/>
+      <c r="BC6" s="25">
+        <f>'0. ГИРА'!BC6</f>
+        <v/>
+      </c>
+      <c r="BD6" s="24" t="n"/>
+      <c r="BE6" s="24" t="n"/>
+      <c r="BF6" s="25">
+        <f>'0. ГИРА'!BF6</f>
+        <v/>
+      </c>
+      <c r="BG6" s="24" t="n"/>
+      <c r="BH6" s="24" t="n"/>
+      <c r="BI6" s="25">
+        <f>'0. ГИРА'!BI6</f>
+        <v/>
+      </c>
+      <c r="BJ6" s="24" t="n"/>
+      <c r="BK6" s="24" t="n"/>
+      <c r="BL6" s="25">
+        <f>'0. ГИРА'!BL6</f>
+        <v/>
+      </c>
+      <c r="BM6" s="24" t="n"/>
+      <c r="BN6" s="24" t="n"/>
+      <c r="BO6" s="25">
+        <f>'0. ГИРА'!BO6</f>
+        <v/>
+      </c>
+      <c r="BP6" s="24" t="n"/>
+      <c r="BQ6" s="24" t="n"/>
+      <c r="BR6" s="25">
+        <f>'0. ГИРА'!BR6</f>
+        <v/>
+      </c>
+      <c r="BS6" s="24" t="n"/>
+      <c r="BT6" s="24" t="n"/>
+      <c r="BU6" s="25">
+        <f>'0. ГИРА'!BU6</f>
+        <v/>
+      </c>
+      <c r="BV6" s="24" t="n"/>
+      <c r="BW6" s="24" t="n"/>
+      <c r="BX6" s="25">
+        <f>'0. ГИРА'!BX6</f>
+        <v/>
+      </c>
+      <c r="BY6" s="24" t="n"/>
+      <c r="BZ6" s="24" t="n"/>
+      <c r="CA6" s="25">
+        <f>'0. ГИРА'!CA6</f>
+        <v/>
+      </c>
+      <c r="CB6" s="24" t="n"/>
+      <c r="CC6" s="24" t="n"/>
+      <c r="CD6" s="25">
+        <f>'0. ГИРА'!CD6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="38" t="inlineStr">
+        <is>
+          <t>Контакт 1</t>
+        </is>
+      </c>
+      <c r="B7" s="33">
+        <f>Реестр!N3</f>
+        <v/>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Водоканал горячая вода</t>
+        </is>
+      </c>
+      <c r="D7" s="67" t="n"/>
+      <c r="E7" s="67" t="n"/>
+      <c r="F7" s="68">
+        <f>E7-D7</f>
+        <v/>
+      </c>
+      <c r="G7" s="69">
+        <f>G8*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="67" t="n"/>
+      <c r="I7" s="68">
+        <f>H7-E7</f>
+        <v/>
+      </c>
+      <c r="J7" s="69">
+        <f>J8*I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="67" t="n"/>
+      <c r="L7" s="68">
+        <f>K7-H7</f>
+        <v/>
+      </c>
+      <c r="M7" s="69">
+        <f>M8*L7</f>
+        <v/>
+      </c>
+      <c r="N7" s="67" t="n"/>
+      <c r="O7" s="68">
+        <f>N7-K7</f>
+        <v/>
+      </c>
+      <c r="P7" s="69">
+        <f>P8*O7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="67" t="n"/>
+      <c r="R7" s="68">
+        <f>Q7-N7</f>
+        <v/>
+      </c>
+      <c r="S7" s="69">
+        <f>S8*R7</f>
+        <v/>
+      </c>
+      <c r="T7" s="67" t="n"/>
+      <c r="U7" s="68">
+        <f>T7-Q7</f>
+        <v/>
+      </c>
+      <c r="V7" s="69">
+        <f>V8*U7</f>
+        <v/>
+      </c>
+      <c r="W7" s="67" t="n"/>
+      <c r="X7" s="68">
+        <f>W7-T7</f>
+        <v/>
+      </c>
+      <c r="Y7" s="69">
+        <f>Y8*X7</f>
+        <v/>
+      </c>
+      <c r="Z7" s="67" t="n"/>
+      <c r="AA7" s="68">
+        <f>Z7-W7</f>
+        <v/>
+      </c>
+      <c r="AB7" s="69">
+        <f>AB8*AA7</f>
+        <v/>
+      </c>
+      <c r="AC7" s="67" t="n"/>
+      <c r="AD7" s="68">
+        <f>AC7-Z7</f>
+        <v/>
+      </c>
+      <c r="AE7" s="69">
+        <f>AE8*AD7</f>
+        <v/>
+      </c>
+      <c r="AF7" s="67" t="n"/>
+      <c r="AG7" s="68">
+        <f>AF7-AC7</f>
+        <v/>
+      </c>
+      <c r="AH7" s="69">
+        <f>AH8*AG7</f>
+        <v/>
+      </c>
+      <c r="AI7" s="67" t="n"/>
+      <c r="AJ7" s="68">
+        <f>AI7-AF7</f>
+        <v/>
+      </c>
+      <c r="AK7" s="69">
+        <f>AK8*AJ7</f>
+        <v/>
+      </c>
+      <c r="AL7" s="67" t="n"/>
+      <c r="AM7" s="68">
+        <f>AL7-AI7</f>
+        <v/>
+      </c>
+      <c r="AN7" s="69">
+        <f>AN8*AM7</f>
+        <v/>
+      </c>
+      <c r="AO7" s="67" t="n"/>
+      <c r="AP7" s="68">
+        <f>AO7-AL7</f>
+        <v/>
+      </c>
+      <c r="AQ7" s="69">
+        <f>AQ8*AP7</f>
+        <v/>
+      </c>
+      <c r="AR7" s="67" t="n"/>
+      <c r="AS7" s="68">
+        <f>AR7-AO7</f>
+        <v/>
+      </c>
+      <c r="AT7" s="69">
+        <f>AT8*AS7</f>
+        <v/>
+      </c>
+      <c r="AU7" s="67" t="n"/>
+      <c r="AV7" s="68">
+        <f>AU7-AR7</f>
+        <v/>
+      </c>
+      <c r="AW7" s="69">
+        <f>AW8*AV7</f>
+        <v/>
+      </c>
+      <c r="AX7" s="67" t="n"/>
+      <c r="AY7" s="68">
+        <f>AX7-AU7</f>
+        <v/>
+      </c>
+      <c r="AZ7" s="69">
+        <f>AZ8*AY7</f>
+        <v/>
+      </c>
+      <c r="BA7" s="67" t="n"/>
+      <c r="BB7" s="68">
+        <f>BA7-AX7</f>
+        <v/>
+      </c>
+      <c r="BC7" s="69">
+        <f>BC8*BB7</f>
+        <v/>
+      </c>
+      <c r="BD7" s="67" t="n"/>
+      <c r="BE7" s="68">
+        <f>BD7-BA7</f>
+        <v/>
+      </c>
+      <c r="BF7" s="69">
+        <f>BF8*BE7</f>
+        <v/>
+      </c>
+      <c r="BG7" s="67" t="n"/>
+      <c r="BH7" s="68">
+        <f>BG7-BD7</f>
+        <v/>
+      </c>
+      <c r="BI7" s="69">
+        <f>BI8*BH7</f>
+        <v/>
+      </c>
+      <c r="BJ7" s="67" t="n"/>
+      <c r="BK7" s="68">
+        <f>BJ7-BG7</f>
+        <v/>
+      </c>
+      <c r="BL7" s="69">
+        <f>BL8*BK7</f>
+        <v/>
+      </c>
+      <c r="BM7" s="67" t="n"/>
+      <c r="BN7" s="68">
+        <f>BM7-BJ7</f>
+        <v/>
+      </c>
+      <c r="BO7" s="69">
+        <f>BO8*BN7</f>
+        <v/>
+      </c>
+      <c r="BP7" s="67" t="n"/>
+      <c r="BQ7" s="68">
+        <f>BP7-BM7</f>
+        <v/>
+      </c>
+      <c r="BR7" s="69">
+        <f>BR8*BQ7</f>
+        <v/>
+      </c>
+      <c r="BS7" s="67" t="n"/>
+      <c r="BT7" s="68">
+        <f>BS7-BP7</f>
+        <v/>
+      </c>
+      <c r="BU7" s="69">
+        <f>BU8*BT7</f>
+        <v/>
+      </c>
+      <c r="BV7" s="67" t="n"/>
+      <c r="BW7" s="68">
+        <f>BV7-BS7</f>
+        <v/>
+      </c>
+      <c r="BX7" s="69">
+        <f>BX8*BW7</f>
+        <v/>
+      </c>
+      <c r="BY7" s="67" t="n"/>
+      <c r="BZ7" s="68">
+        <f>BY7-BV7</f>
+        <v/>
+      </c>
+      <c r="CA7" s="69">
+        <f>CA8*BZ7</f>
+        <v/>
+      </c>
+      <c r="CB7" s="67" t="n"/>
+      <c r="CC7" s="68">
+        <f>CB7-BY7</f>
+        <v/>
+      </c>
+      <c r="CD7" s="69">
+        <f>CD8*CC7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>Имя 2</t>
+        </is>
+      </c>
+      <c r="B8" s="34">
+        <f>Реестр!O3</f>
+        <v/>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Водоканал горячая Тариф</t>
+        </is>
+      </c>
+      <c r="D8" s="70" t="n"/>
+      <c r="E8" s="70" t="n"/>
+      <c r="F8" s="70" t="n"/>
+      <c r="G8" s="71">
+        <f>'0. ГИРА'!G8</f>
+        <v/>
+      </c>
+      <c r="H8" s="70" t="n"/>
+      <c r="I8" s="70" t="n"/>
+      <c r="J8" s="71">
+        <f>'0. ГИРА'!J8</f>
+        <v/>
+      </c>
+      <c r="K8" s="70" t="n"/>
+      <c r="L8" s="70" t="n"/>
+      <c r="M8" s="71">
+        <f>'0. ГИРА'!M8</f>
+        <v/>
+      </c>
+      <c r="N8" s="70" t="n"/>
+      <c r="O8" s="70" t="n"/>
+      <c r="P8" s="71">
+        <f>'0. ГИРА'!P8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="70" t="n"/>
+      <c r="R8" s="70" t="n"/>
+      <c r="S8" s="71">
+        <f>'0. ГИРА'!S8</f>
+        <v/>
+      </c>
+      <c r="T8" s="70" t="n"/>
+      <c r="U8" s="70" t="n"/>
+      <c r="V8" s="71">
+        <f>'0. ГИРА'!V8</f>
+        <v/>
+      </c>
+      <c r="W8" s="70" t="n"/>
+      <c r="X8" s="70" t="n"/>
+      <c r="Y8" s="71">
+        <f>'0. ГИРА'!Y8</f>
+        <v/>
+      </c>
+      <c r="Z8" s="70" t="n"/>
+      <c r="AA8" s="70" t="n"/>
+      <c r="AB8" s="71">
+        <f>'0. ГИРА'!AB8</f>
+        <v/>
+      </c>
+      <c r="AC8" s="70" t="n"/>
+      <c r="AD8" s="70" t="n"/>
+      <c r="AE8" s="71">
+        <f>'0. ГИРА'!AE8</f>
+        <v/>
+      </c>
+      <c r="AF8" s="70" t="n"/>
+      <c r="AG8" s="70" t="n"/>
+      <c r="AH8" s="71">
+        <f>'0. ГИРА'!AH8</f>
+        <v/>
+      </c>
+      <c r="AI8" s="70" t="n"/>
+      <c r="AJ8" s="70" t="n"/>
+      <c r="AK8" s="71">
+        <f>'0. ГИРА'!AK8</f>
+        <v/>
+      </c>
+      <c r="AL8" s="70" t="n"/>
+      <c r="AM8" s="70" t="n"/>
+      <c r="AN8" s="71">
+        <f>'0. ГИРА'!AN8</f>
+        <v/>
+      </c>
+      <c r="AO8" s="70" t="n"/>
+      <c r="AP8" s="70" t="n"/>
+      <c r="AQ8" s="71">
+        <f>'0. ГИРА'!AQ8</f>
+        <v/>
+      </c>
+      <c r="AR8" s="70" t="n"/>
+      <c r="AS8" s="70" t="n"/>
+      <c r="AT8" s="71">
+        <f>'0. ГИРА'!AT8</f>
+        <v/>
+      </c>
+      <c r="AU8" s="70" t="n"/>
+      <c r="AV8" s="70" t="n"/>
+      <c r="AW8" s="71">
+        <f>'0. ГИРА'!AW8</f>
+        <v/>
+      </c>
+      <c r="AX8" s="70" t="n"/>
+      <c r="AY8" s="70" t="n"/>
+      <c r="AZ8" s="71">
+        <f>'0. ГИРА'!AZ8</f>
+        <v/>
+      </c>
+      <c r="BA8" s="70" t="n"/>
+      <c r="BB8" s="70" t="n"/>
+      <c r="BC8" s="71">
+        <f>'0. ГИРА'!BC8</f>
+        <v/>
+      </c>
+      <c r="BD8" s="70" t="n"/>
+      <c r="BE8" s="70" t="n"/>
+      <c r="BF8" s="71">
+        <f>'0. ГИРА'!BF8</f>
+        <v/>
+      </c>
+      <c r="BG8" s="70" t="n"/>
+      <c r="BH8" s="70" t="n"/>
+      <c r="BI8" s="71">
+        <f>'0. ГИРА'!BI8</f>
+        <v/>
+      </c>
+      <c r="BJ8" s="70" t="n"/>
+      <c r="BK8" s="70" t="n"/>
+      <c r="BL8" s="71">
+        <f>'0. ГИРА'!BL8</f>
+        <v/>
+      </c>
+      <c r="BM8" s="70" t="n"/>
+      <c r="BN8" s="70" t="n"/>
+      <c r="BO8" s="71">
+        <f>'0. ГИРА'!BO8</f>
+        <v/>
+      </c>
+      <c r="BP8" s="70" t="n"/>
+      <c r="BQ8" s="70" t="n"/>
+      <c r="BR8" s="71">
+        <f>'0. ГИРА'!BR8</f>
+        <v/>
+      </c>
+      <c r="BS8" s="70" t="n"/>
+      <c r="BT8" s="70" t="n"/>
+      <c r="BU8" s="71">
+        <f>'0. ГИРА'!BU8</f>
+        <v/>
+      </c>
+      <c r="BV8" s="70" t="n"/>
+      <c r="BW8" s="70" t="n"/>
+      <c r="BX8" s="71">
+        <f>'0. ГИРА'!BX8</f>
+        <v/>
+      </c>
+      <c r="BY8" s="70" t="n"/>
+      <c r="BZ8" s="70" t="n"/>
+      <c r="CA8" s="71">
+        <f>'0. ГИРА'!CA8</f>
+        <v/>
+      </c>
+      <c r="CB8" s="70" t="n"/>
+      <c r="CC8" s="70" t="n"/>
+      <c r="CD8" s="71">
+        <f>'0. ГИРА'!CD8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>Контакт 2</t>
+        </is>
+      </c>
+      <c r="B9" s="33">
+        <f>Реестр!P3</f>
+        <v/>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Тепло</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="22">
+        <f>E9-D9</f>
+        <v/>
+      </c>
+      <c r="G9" s="23">
+        <f>G10*B3</f>
+        <v/>
+      </c>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="22">
+        <f>H9-E9</f>
+        <v/>
+      </c>
+      <c r="J9" s="23">
+        <f>J10*E3</f>
+        <v/>
+      </c>
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="22">
+        <f>K9-H9</f>
+        <v/>
+      </c>
+      <c r="M9" s="23">
+        <f>M10*H3</f>
+        <v/>
+      </c>
+      <c r="N9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="22">
+        <f>N9-K9</f>
+        <v/>
+      </c>
+      <c r="P9" s="23" t="n">
+        <v>21214</v>
+      </c>
+      <c r="Q9" s="21" t="n"/>
+      <c r="R9" s="22">
+        <f>Q9-N9</f>
+        <v/>
+      </c>
+      <c r="S9" s="23">
+        <f>S10*N3</f>
+        <v/>
+      </c>
+      <c r="T9" s="21" t="n"/>
+      <c r="U9" s="22">
+        <f>T9-Q9</f>
+        <v/>
+      </c>
+      <c r="V9" s="23">
+        <f>V10*Q3</f>
+        <v/>
+      </c>
+      <c r="W9" s="21" t="n"/>
+      <c r="X9" s="22">
+        <f>W9-T9</f>
+        <v/>
+      </c>
+      <c r="Y9" s="23">
+        <f>Y10*T3</f>
+        <v/>
+      </c>
+      <c r="Z9" s="21" t="n"/>
+      <c r="AA9" s="22">
+        <f>Z9-W9</f>
+        <v/>
+      </c>
+      <c r="AB9" s="23">
+        <f>AB10*W3</f>
+        <v/>
+      </c>
+      <c r="AC9" s="21" t="n"/>
+      <c r="AD9" s="22">
+        <f>AC9-Z9</f>
+        <v/>
+      </c>
+      <c r="AE9" s="23">
+        <f>AE10*Z3</f>
+        <v/>
+      </c>
+      <c r="AF9" s="21" t="n"/>
+      <c r="AG9" s="22">
+        <f>AF9-AC9</f>
+        <v/>
+      </c>
+      <c r="AH9" s="23">
+        <f>AH10*AC3</f>
+        <v/>
+      </c>
+      <c r="AI9" s="21" t="n"/>
+      <c r="AJ9" s="22">
+        <f>AI9-AF9</f>
+        <v/>
+      </c>
+      <c r="AK9" s="23">
+        <f>AK10*AF3</f>
+        <v/>
+      </c>
+      <c r="AL9" s="21" t="n"/>
+      <c r="AM9" s="22">
+        <f>AL9-AI9</f>
+        <v/>
+      </c>
+      <c r="AN9" s="23">
+        <f>AN10*AI3</f>
+        <v/>
+      </c>
+      <c r="AO9" s="21" t="n"/>
+      <c r="AP9" s="22">
+        <f>AO9-AL9</f>
+        <v/>
+      </c>
+      <c r="AQ9" s="23">
+        <f>AQ10*AL3</f>
+        <v/>
+      </c>
+      <c r="AR9" s="21" t="n"/>
+      <c r="AS9" s="22">
+        <f>AR9-AO9</f>
+        <v/>
+      </c>
+      <c r="AT9" s="23">
+        <f>AT10*AO3</f>
+        <v/>
+      </c>
+      <c r="AU9" s="21" t="n"/>
+      <c r="AV9" s="22">
+        <f>AU9-AR9</f>
+        <v/>
+      </c>
+      <c r="AW9" s="23">
+        <f>AW10*AR3</f>
+        <v/>
+      </c>
+      <c r="AX9" s="21" t="n"/>
+      <c r="AY9" s="22">
+        <f>AX9-AU9</f>
+        <v/>
+      </c>
+      <c r="AZ9" s="23">
+        <f>AZ10*AU3</f>
+        <v/>
+      </c>
+      <c r="BA9" s="21" t="n"/>
+      <c r="BB9" s="22">
+        <f>BA9-AX9</f>
+        <v/>
+      </c>
+      <c r="BC9" s="23">
+        <f>BC10*AX3</f>
+        <v/>
+      </c>
+      <c r="BD9" s="21" t="n"/>
+      <c r="BE9" s="22">
+        <f>BD9-BA9</f>
+        <v/>
+      </c>
+      <c r="BF9" s="23">
+        <f>BF10*BA3</f>
+        <v/>
+      </c>
+      <c r="BG9" s="21" t="n"/>
+      <c r="BH9" s="22">
+        <f>BG9-BD9</f>
+        <v/>
+      </c>
+      <c r="BI9" s="23">
+        <f>BI10*BD3</f>
+        <v/>
+      </c>
+      <c r="BJ9" s="21" t="n"/>
+      <c r="BK9" s="22">
+        <f>BJ9-BG9</f>
+        <v/>
+      </c>
+      <c r="BL9" s="23">
+        <f>BL10*BG3</f>
+        <v/>
+      </c>
+      <c r="BM9" s="21" t="n"/>
+      <c r="BN9" s="22">
+        <f>BM9-BJ9</f>
+        <v/>
+      </c>
+      <c r="BO9" s="23">
+        <f>BO10*BJ3</f>
+        <v/>
+      </c>
+      <c r="BP9" s="21" t="n"/>
+      <c r="BQ9" s="22">
+        <f>BP9-BM9</f>
+        <v/>
+      </c>
+      <c r="BR9" s="23">
+        <f>BR10*BM3</f>
+        <v/>
+      </c>
+      <c r="BS9" s="21" t="n"/>
+      <c r="BT9" s="22">
+        <f>BS9-BP9</f>
+        <v/>
+      </c>
+      <c r="BU9" s="23">
+        <f>BU10*BP3</f>
+        <v/>
+      </c>
+      <c r="BV9" s="21" t="n"/>
+      <c r="BW9" s="22">
+        <f>BV9-BS9</f>
+        <v/>
+      </c>
+      <c r="BX9" s="23">
+        <f>BX10*BS3</f>
+        <v/>
+      </c>
+      <c r="BY9" s="21" t="n"/>
+      <c r="BZ9" s="22">
+        <f>BY9-BV9</f>
+        <v/>
+      </c>
+      <c r="CA9" s="23">
+        <f>CA10*BV3</f>
+        <v/>
+      </c>
+      <c r="CB9" s="21" t="n"/>
+      <c r="CC9" s="22">
+        <f>CB9-BY9</f>
+        <v/>
+      </c>
+      <c r="CD9" s="23">
+        <f>CD10*BY3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Тепло тариф</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="25">
+        <f>'0. ГИРА'!G10</f>
+        <v/>
+      </c>
+      <c r="H10" s="24" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="25">
+        <f>'0. ГИРА'!J10</f>
+        <v/>
+      </c>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="24" t="n"/>
+      <c r="M10" s="25">
+        <f>'0. ГИРА'!M10</f>
+        <v/>
+      </c>
+      <c r="N10" s="24" t="n"/>
+      <c r="O10" s="24" t="n"/>
+      <c r="P10" s="25">
+        <f>'0. ГИРА'!P10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="24" t="n"/>
+      <c r="R10" s="24" t="n"/>
+      <c r="S10" s="25">
+        <f>'0. ГИРА'!S10</f>
+        <v/>
+      </c>
+      <c r="T10" s="24" t="n"/>
+      <c r="U10" s="24" t="n"/>
+      <c r="V10" s="25">
+        <f>'0. ГИРА'!V10</f>
+        <v/>
+      </c>
+      <c r="W10" s="24" t="n"/>
+      <c r="X10" s="24" t="n"/>
+      <c r="Y10" s="25">
+        <f>'0. ГИРА'!Y10</f>
+        <v/>
+      </c>
+      <c r="Z10" s="24" t="n"/>
+      <c r="AA10" s="24" t="n"/>
+      <c r="AB10" s="25">
+        <f>'0. ГИРА'!AB10</f>
+        <v/>
+      </c>
+      <c r="AC10" s="24" t="n"/>
+      <c r="AD10" s="24" t="n"/>
+      <c r="AE10" s="25">
+        <f>'0. ГИРА'!AE10</f>
+        <v/>
+      </c>
+      <c r="AF10" s="24" t="n"/>
+      <c r="AG10" s="24" t="n"/>
+      <c r="AH10" s="25">
+        <f>'0. ГИРА'!AH10</f>
+        <v/>
+      </c>
+      <c r="AI10" s="24" t="n"/>
+      <c r="AJ10" s="24" t="n"/>
+      <c r="AK10" s="25">
+        <f>'0. ГИРА'!AK10</f>
+        <v/>
+      </c>
+      <c r="AL10" s="24" t="n"/>
+      <c r="AM10" s="24" t="n"/>
+      <c r="AN10" s="25">
+        <f>'0. ГИРА'!AN10</f>
+        <v/>
+      </c>
+      <c r="AO10" s="24" t="n"/>
+      <c r="AP10" s="24" t="n"/>
+      <c r="AQ10" s="25">
+        <f>'0. ГИРА'!AQ10</f>
+        <v/>
+      </c>
+      <c r="AR10" s="24" t="n"/>
+      <c r="AS10" s="24" t="n"/>
+      <c r="AT10" s="25">
+        <f>'0. ГИРА'!AT10</f>
+        <v/>
+      </c>
+      <c r="AU10" s="24" t="n"/>
+      <c r="AV10" s="24" t="n"/>
+      <c r="AW10" s="25">
+        <f>'0. ГИРА'!AW10</f>
+        <v/>
+      </c>
+      <c r="AX10" s="24" t="n"/>
+      <c r="AY10" s="24" t="n"/>
+      <c r="AZ10" s="25">
+        <f>'0. ГИРА'!AZ10</f>
+        <v/>
+      </c>
+      <c r="BA10" s="24" t="n"/>
+      <c r="BB10" s="24" t="n"/>
+      <c r="BC10" s="25">
+        <f>'0. ГИРА'!BC10</f>
+        <v/>
+      </c>
+      <c r="BD10" s="24" t="n"/>
+      <c r="BE10" s="24" t="n"/>
+      <c r="BF10" s="25">
+        <f>'0. ГИРА'!BF10</f>
+        <v/>
+      </c>
+      <c r="BG10" s="24" t="n"/>
+      <c r="BH10" s="24" t="n"/>
+      <c r="BI10" s="25">
+        <f>'0. ГИРА'!BI10</f>
+        <v/>
+      </c>
+      <c r="BJ10" s="24" t="n"/>
+      <c r="BK10" s="24" t="n"/>
+      <c r="BL10" s="25">
+        <f>'0. ГИРА'!BL10</f>
+        <v/>
+      </c>
+      <c r="BM10" s="24" t="n"/>
+      <c r="BN10" s="24" t="n"/>
+      <c r="BO10" s="25">
+        <f>'0. ГИРА'!BO10</f>
+        <v/>
+      </c>
+      <c r="BP10" s="24" t="n"/>
+      <c r="BQ10" s="24" t="n"/>
+      <c r="BR10" s="25">
+        <f>'0. ГИРА'!BR10</f>
+        <v/>
+      </c>
+      <c r="BS10" s="24" t="n"/>
+      <c r="BT10" s="24" t="n"/>
+      <c r="BU10" s="25">
+        <f>'0. ГИРА'!BU10</f>
+        <v/>
+      </c>
+      <c r="BV10" s="24" t="n"/>
+      <c r="BW10" s="24" t="n"/>
+      <c r="BX10" s="25">
+        <f>'0. ГИРА'!BX10</f>
+        <v/>
+      </c>
+      <c r="BY10" s="24" t="n"/>
+      <c r="BZ10" s="24" t="n"/>
+      <c r="CA10" s="25">
+        <f>'0. ГИРА'!CA10</f>
+        <v/>
+      </c>
+      <c r="CB10" s="24" t="n"/>
+      <c r="CC10" s="24" t="n"/>
+      <c r="CD10" s="25">
+        <f>'0. ГИРА'!CD10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="66" t="inlineStr">
+        <is>
+          <t>Номер счетчика</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 43432,34343</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Экспл. Услуги от УК</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="22">
+        <f>E11-D11</f>
+        <v/>
+      </c>
+      <c r="G11" s="23">
+        <f>'0. ГИРА'!G12</f>
+        <v/>
+      </c>
+      <c r="H11" s="21" t="n"/>
+      <c r="I11" s="22">
+        <f>H11-E11</f>
+        <v/>
+      </c>
+      <c r="J11" s="23">
+        <f>'0. ГИРА'!J12</f>
+        <v/>
+      </c>
+      <c r="K11" s="21" t="n"/>
+      <c r="L11" s="22">
+        <f>K11-H11</f>
+        <v/>
+      </c>
+      <c r="M11" s="23">
+        <f>'0. ГИРА'!M12</f>
+        <v/>
+      </c>
+      <c r="N11" s="21" t="n"/>
+      <c r="O11" s="22">
+        <f>N11-K11</f>
+        <v/>
+      </c>
+      <c r="P11" s="23">
+        <f>'0. ГИРА'!P12</f>
+        <v/>
+      </c>
+      <c r="Q11" s="21" t="n"/>
+      <c r="R11" s="22">
+        <f>Q11-N11</f>
+        <v/>
+      </c>
+      <c r="S11" s="23">
+        <f>'0. ГИРА'!S12</f>
+        <v/>
+      </c>
+      <c r="T11" s="21" t="n"/>
+      <c r="U11" s="22">
+        <f>T11-Q11</f>
+        <v/>
+      </c>
+      <c r="V11" s="23">
+        <f>'0. ГИРА'!V12</f>
+        <v/>
+      </c>
+      <c r="W11" s="21" t="n"/>
+      <c r="X11" s="22">
+        <f>W11-T11</f>
+        <v/>
+      </c>
+      <c r="Y11" s="23">
+        <f>'0. ГИРА'!Y12</f>
+        <v/>
+      </c>
+      <c r="Z11" s="21" t="n"/>
+      <c r="AA11" s="22">
+        <f>Z11-W11</f>
+        <v/>
+      </c>
+      <c r="AB11" s="23">
+        <f>'0. ГИРА'!AB12</f>
+        <v/>
+      </c>
+      <c r="AC11" s="21" t="n"/>
+      <c r="AD11" s="22">
+        <f>AC11-Z11</f>
+        <v/>
+      </c>
+      <c r="AE11" s="23">
+        <f>'0. ГИРА'!AE12</f>
+        <v/>
+      </c>
+      <c r="AF11" s="21" t="n"/>
+      <c r="AG11" s="22">
+        <f>AF11-AC11</f>
+        <v/>
+      </c>
+      <c r="AH11" s="23">
+        <f>'0. ГИРА'!AH12</f>
+        <v/>
+      </c>
+      <c r="AI11" s="21" t="n"/>
+      <c r="AJ11" s="22">
+        <f>AI11-AF11</f>
+        <v/>
+      </c>
+      <c r="AK11" s="23">
+        <f>'0. ГИРА'!AK12</f>
+        <v/>
+      </c>
+      <c r="AL11" s="21" t="n"/>
+      <c r="AM11" s="22">
+        <f>AL11-AI11</f>
+        <v/>
+      </c>
+      <c r="AN11" s="23">
+        <f>'0. ГИРА'!AN12</f>
+        <v/>
+      </c>
+      <c r="AO11" s="21" t="n"/>
+      <c r="AP11" s="22">
+        <f>AO11-AL11</f>
+        <v/>
+      </c>
+      <c r="AQ11" s="23">
+        <f>'0. ГИРА'!AQ12</f>
+        <v/>
+      </c>
+      <c r="AR11" s="21" t="n"/>
+      <c r="AS11" s="22">
+        <f>AR11-AO11</f>
+        <v/>
+      </c>
+      <c r="AT11" s="23">
+        <f>'0. ГИРА'!AT12</f>
+        <v/>
+      </c>
+      <c r="AU11" s="21" t="n"/>
+      <c r="AV11" s="22">
+        <f>AU11-AR11</f>
+        <v/>
+      </c>
+      <c r="AW11" s="23">
+        <f>'0. ГИРА'!AW12</f>
+        <v/>
+      </c>
+      <c r="AX11" s="21" t="n"/>
+      <c r="AY11" s="22">
+        <f>AX11-AU11</f>
+        <v/>
+      </c>
+      <c r="AZ11" s="23">
+        <f>'0. ГИРА'!AZ12</f>
+        <v/>
+      </c>
+      <c r="BA11" s="21" t="n"/>
+      <c r="BB11" s="22">
+        <f>BA11-AX11</f>
+        <v/>
+      </c>
+      <c r="BC11" s="23">
+        <f>'0. ГИРА'!BC12</f>
+        <v/>
+      </c>
+      <c r="BD11" s="21" t="n"/>
+      <c r="BE11" s="22">
+        <f>BD11-BA11</f>
+        <v/>
+      </c>
+      <c r="BF11" s="23">
+        <f>'0. ГИРА'!BF12</f>
+        <v/>
+      </c>
+      <c r="BG11" s="21" t="n"/>
+      <c r="BH11" s="22">
+        <f>BG11-BD11</f>
+        <v/>
+      </c>
+      <c r="BI11" s="23">
+        <f>'0. ГИРА'!BI12</f>
+        <v/>
+      </c>
+      <c r="BJ11" s="21" t="n"/>
+      <c r="BK11" s="22">
+        <f>BJ11-BG11</f>
+        <v/>
+      </c>
+      <c r="BL11" s="23">
+        <f>'0. ГИРА'!BL12</f>
+        <v/>
+      </c>
+      <c r="BM11" s="21" t="n"/>
+      <c r="BN11" s="22">
+        <f>BM11-BJ11</f>
+        <v/>
+      </c>
+      <c r="BO11" s="23">
+        <f>'0. ГИРА'!BO12</f>
+        <v/>
+      </c>
+      <c r="BP11" s="21" t="n"/>
+      <c r="BQ11" s="22">
+        <f>BP11-BM11</f>
+        <v/>
+      </c>
+      <c r="BR11" s="23">
+        <f>'0. ГИРА'!BR12</f>
+        <v/>
+      </c>
+      <c r="BS11" s="21" t="n"/>
+      <c r="BT11" s="22">
+        <f>BS11-BP11</f>
+        <v/>
+      </c>
+      <c r="BU11" s="23">
+        <f>'0. ГИРА'!BU12</f>
+        <v/>
+      </c>
+      <c r="BV11" s="21" t="n"/>
+      <c r="BW11" s="22">
+        <f>BV11-BS11</f>
+        <v/>
+      </c>
+      <c r="BX11" s="23">
+        <f>'0. ГИРА'!BX12</f>
+        <v/>
+      </c>
+      <c r="BY11" s="21" t="n"/>
+      <c r="BZ11" s="22">
+        <f>BY11-BV11</f>
+        <v/>
+      </c>
+      <c r="CA11" s="23">
+        <f>'0. ГИРА'!CA12</f>
+        <v/>
+      </c>
+      <c r="CB11" s="21" t="n"/>
+      <c r="CC11" s="22">
+        <f>CB11-BY11</f>
+        <v/>
+      </c>
+      <c r="CD11" s="23">
+        <f>'0. ГИРА'!CD12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Экспл. Услуги от УК тариф</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="24" t="n"/>
+      <c r="G12" s="25">
+        <f>'0. ГИРА'!G12</f>
+        <v/>
+      </c>
+      <c r="H12" s="24" t="n"/>
+      <c r="I12" s="24" t="n"/>
+      <c r="J12" s="25">
+        <f>'0. ГИРА'!J12</f>
+        <v/>
+      </c>
+      <c r="K12" s="24" t="n"/>
+      <c r="L12" s="24" t="n"/>
+      <c r="M12" s="25">
+        <f>'0. ГИРА'!M12</f>
+        <v/>
+      </c>
+      <c r="N12" s="24" t="n"/>
+      <c r="O12" s="24" t="n"/>
+      <c r="P12" s="25" t="n">
+        <v>421412</v>
+      </c>
+      <c r="Q12" s="24" t="n"/>
+      <c r="R12" s="24" t="n"/>
+      <c r="S12" s="25">
+        <f>'0. ГИРА'!S12</f>
+        <v/>
+      </c>
+      <c r="T12" s="24" t="n"/>
+      <c r="U12" s="24" t="n"/>
+      <c r="V12" s="25">
+        <f>'0. ГИРА'!V12</f>
+        <v/>
+      </c>
+      <c r="W12" s="24" t="n"/>
+      <c r="X12" s="24" t="n"/>
+      <c r="Y12" s="25">
+        <f>'0. ГИРА'!Y12</f>
+        <v/>
+      </c>
+      <c r="Z12" s="24" t="n"/>
+      <c r="AA12" s="24" t="n"/>
+      <c r="AB12" s="25">
+        <f>'0. ГИРА'!AB12</f>
+        <v/>
+      </c>
+      <c r="AC12" s="24" t="n"/>
+      <c r="AD12" s="24" t="n"/>
+      <c r="AE12" s="25">
+        <f>'0. ГИРА'!AE12</f>
+        <v/>
+      </c>
+      <c r="AF12" s="24" t="n"/>
+      <c r="AG12" s="24" t="n"/>
+      <c r="AH12" s="25">
+        <f>'0. ГИРА'!AH12</f>
+        <v/>
+      </c>
+      <c r="AI12" s="24" t="n"/>
+      <c r="AJ12" s="24" t="n"/>
+      <c r="AK12" s="25">
+        <f>'0. ГИРА'!AK12</f>
+        <v/>
+      </c>
+      <c r="AL12" s="24" t="n"/>
+      <c r="AM12" s="24" t="n"/>
+      <c r="AN12" s="25">
+        <f>'0. ГИРА'!AN12</f>
+        <v/>
+      </c>
+      <c r="AO12" s="24" t="n"/>
+      <c r="AP12" s="24" t="n"/>
+      <c r="AQ12" s="25">
+        <f>'0. ГИРА'!AQ12</f>
+        <v/>
+      </c>
+      <c r="AR12" s="24" t="n"/>
+      <c r="AS12" s="24" t="n"/>
+      <c r="AT12" s="25">
+        <f>'0. ГИРА'!AT12</f>
+        <v/>
+      </c>
+      <c r="AU12" s="24" t="n"/>
+      <c r="AV12" s="24" t="n"/>
+      <c r="AW12" s="25">
+        <f>'0. ГИРА'!AW12</f>
+        <v/>
+      </c>
+      <c r="AX12" s="24" t="n"/>
+      <c r="AY12" s="24" t="n"/>
+      <c r="AZ12" s="25">
+        <f>'0. ГИРА'!AZ12</f>
+        <v/>
+      </c>
+      <c r="BA12" s="24" t="n"/>
+      <c r="BB12" s="24" t="n"/>
+      <c r="BC12" s="25">
+        <f>'0. ГИРА'!BC12</f>
+        <v/>
+      </c>
+      <c r="BD12" s="24" t="n"/>
+      <c r="BE12" s="24" t="n"/>
+      <c r="BF12" s="25">
+        <f>'0. ГИРА'!BF12</f>
+        <v/>
+      </c>
+      <c r="BG12" s="24" t="n"/>
+      <c r="BH12" s="24" t="n"/>
+      <c r="BI12" s="25">
+        <f>'0. ГИРА'!BI12</f>
+        <v/>
+      </c>
+      <c r="BJ12" s="24" t="n"/>
+      <c r="BK12" s="24" t="n"/>
+      <c r="BL12" s="25">
+        <f>'0. ГИРА'!BL12</f>
+        <v/>
+      </c>
+      <c r="BM12" s="24" t="n"/>
+      <c r="BN12" s="24" t="n"/>
+      <c r="BO12" s="25">
+        <f>'0. ГИРА'!BO12</f>
+        <v/>
+      </c>
+      <c r="BP12" s="24" t="n"/>
+      <c r="BQ12" s="24" t="n"/>
+      <c r="BR12" s="25">
+        <f>'0. ГИРА'!BR12</f>
+        <v/>
+      </c>
+      <c r="BS12" s="24" t="n"/>
+      <c r="BT12" s="24" t="n"/>
+      <c r="BU12" s="25">
+        <f>'0. ГИРА'!BU12</f>
+        <v/>
+      </c>
+      <c r="BV12" s="24" t="n"/>
+      <c r="BW12" s="24" t="n"/>
+      <c r="BX12" s="25">
+        <f>'0. ГИРА'!BX12</f>
+        <v/>
+      </c>
+      <c r="BY12" s="24" t="n"/>
+      <c r="BZ12" s="24" t="n"/>
+      <c r="CA12" s="25">
+        <f>'0. ГИРА'!CA12</f>
+        <v/>
+      </c>
+      <c r="CB12" s="24" t="n"/>
+      <c r="CC12" s="24" t="n"/>
+      <c r="CD12" s="25">
+        <f>'0. ГИРА'!CD12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="16" t="n"/>
+      <c r="P13" t="n">
+        <v>4124124</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" s="16" t="n"/>
+    </row>
+    <row r="15">
+      <c r="G15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="G16" s="16" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>